<commit_message>
Stylistic changes for the main.cpp file
</commit_message>
<xml_diff>
--- a/Pomiary.xlsx
+++ b/Pomiary.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a3eea4af91086274/Pulpit/SBD/P1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a3eea4af91086274/Pulpit/SEM5/SBD/P1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2FCF4A24-72F7-4805-86B8-F02B7F7B739A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{2FCF4A24-72F7-4805-86B8-F02B7F7B739A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B432F5D7-AA74-47C7-A04E-2FA9670C920D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{63E0899F-1F7B-41C1-81BE-D2DEB1B2E785}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{63E0899F-1F7B-41C1-81BE-D2DEB1B2E785}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -76,7 +76,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="#,##0.00\ _z_ł"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00\ _z_ł"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -113,7 +113,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -253,46 +253,46 @@
                   <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>25</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>27</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>63</c:v>
+                  <c:v>58</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>100</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>231</c:v>
+                  <c:v>214</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>446</c:v>
+                  <c:v>444</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>985</c:v>
+                  <c:v>926</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>2014</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>4439</c:v>
+                  <c:v>4186</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>9078</c:v>
+                  <c:v>9074</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>19929</c:v>
+                  <c:v>18914</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>40630</c:v>
+                  <c:v>40634</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>88565</c:v>
+                  <c:v>84466</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>179618</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1590,15 +1590,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0FACBD2-E050-4C25-B7F3-B372F54F54CB}">
   <dimension ref="A1:K16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="5" width="8.88671875" style="1"/>
-    <col min="6" max="6" width="12.88671875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" style="2" customWidth="1"/>
+    <col min="2" max="5" width="8.85546875" style="1"/>
+    <col min="6" max="6" width="12.85546875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" style="2" customWidth="1"/>
     <col min="8" max="8" width="13" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>256</v>
       </c>
@@ -1655,11 +1655,11 @@
         <v>3.1</v>
       </c>
       <c r="G2" s="2">
-        <f>(2*B2/$A$2)*(1.04*LOG(B2/2,2)+1.5+IF(MOD(ROUND(K2,0)-1,3)=0,0,1))</f>
+        <f t="shared" ref="G2:G16" si="0">(2*B2/$A$2)*(1.04*LOG(B2/2,2)+1.5+IF(MOD(ROUND(K2,0)-1,3)=0,0,1))</f>
         <v>3.35</v>
       </c>
       <c r="H2" s="1">
-        <f>(E2-F2)/E2</f>
+        <f t="shared" ref="H2:H16" si="1">(E2-F2)/E2</f>
         <v>0.83684210526315794</v>
       </c>
       <c r="I2" s="1">
@@ -1674,45 +1674,45 @@
         <v>7.1999999999999993</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1">
         <v>128</v>
       </c>
       <c r="C3" s="1">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" s="1">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3" s="1">
         <f>SUM(C3:D3)</f>
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F3" s="2">
-        <f t="shared" ref="F3:F16" si="0">(2*B3/$A$2)*(1.04*LOG(B3/2,2)+1)</f>
+        <f t="shared" ref="F3:F16" si="2">(2*B3/$A$2)*(1.04*LOG(B3/2,2)+1)</f>
         <v>7.24</v>
       </c>
       <c r="G3" s="2">
-        <f>(2*B3/$A$2)*(1.04*LOG(B3/2,2)+1.5+IF(MOD(ROUND(K3,0)-1,3)=0,0,1))</f>
+        <f t="shared" si="0"/>
         <v>8.74</v>
       </c>
       <c r="H3" s="1">
-        <f>(E3-F3)/E3</f>
-        <v>0.71039999999999992</v>
+        <f t="shared" si="1"/>
+        <v>0.68521739130434778</v>
       </c>
       <c r="I3" s="1">
-        <f t="shared" ref="I3:I16" si="1">(E3-G3)/E3</f>
-        <v>0.65039999999999987</v>
+        <f t="shared" ref="I3:I16" si="3">(E3-G3)/E3</f>
+        <v>0.62</v>
       </c>
       <c r="J3" s="1">
         <v>9</v>
       </c>
       <c r="K3" s="1">
-        <f t="shared" ref="K3:K16" si="2">1.44*LOG(B3/2,2)</f>
+        <f t="shared" ref="K3:K16" si="4">1.44*LOG(B3/2,2)</f>
         <v>8.64</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B4" s="1">
         <v>256</v>
       </c>
@@ -1723,72 +1723,72 @@
         <v>12</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" ref="E4:E16" si="3">SUM(C4:D4)</f>
+        <f t="shared" ref="E4:E16" si="5">SUM(C4:D4)</f>
         <v>27</v>
       </c>
       <c r="F4" s="2">
+        <f t="shared" si="2"/>
+        <v>16.560000000000002</v>
+      </c>
+      <c r="G4" s="2">
         <f t="shared" si="0"/>
-        <v>16.560000000000002</v>
-      </c>
-      <c r="G4" s="2">
-        <f>(2*B4/$A$2)*(1.04*LOG(B4/2,2)+1.5+IF(MOD(ROUND(K4,0)-1,3)=0,0,1))</f>
         <v>17.560000000000002</v>
       </c>
       <c r="H4" s="1">
-        <f>(E4-F4)/E4</f>
+        <f t="shared" si="1"/>
         <v>0.3866666666666666</v>
       </c>
       <c r="I4" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.34962962962962957</v>
       </c>
       <c r="J4" s="1">
         <v>10</v>
       </c>
       <c r="K4" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>10.08</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>512</v>
       </c>
       <c r="C5" s="1">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D5" s="1">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1">
+        <f t="shared" si="5"/>
+        <v>58</v>
+      </c>
+      <c r="F5" s="2">
+        <f t="shared" si="2"/>
+        <v>37.28</v>
+      </c>
+      <c r="G5" s="2">
+        <f t="shared" si="0"/>
+        <v>43.28</v>
+      </c>
+      <c r="H5" s="1">
+        <f t="shared" si="1"/>
+        <v>0.35724137931034483</v>
+      </c>
+      <c r="I5" s="1">
         <f t="shared" si="3"/>
-        <v>63</v>
-      </c>
-      <c r="F5" s="2">
-        <f t="shared" si="0"/>
-        <v>37.28</v>
-      </c>
-      <c r="G5" s="2">
-        <f>(2*B5/$A$2)*(1.04*LOG(B5/2,2)+1.5+IF(MOD(ROUND(K5,0)-1,3)=0,0,1))</f>
-        <v>43.28</v>
-      </c>
-      <c r="H5" s="1">
-        <f>(E5-F5)/E5</f>
-        <v>0.40825396825396826</v>
-      </c>
-      <c r="I5" s="1">
-        <f t="shared" si="1"/>
-        <v>0.31301587301587303</v>
+        <v>0.25379310344827583</v>
       </c>
       <c r="J5" s="1">
         <v>12</v>
       </c>
       <c r="K5" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>11.52</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>1024</v>
       </c>
@@ -1799,11 +1799,11 @@
         <v>47</v>
       </c>
       <c r="E6" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>100</v>
       </c>
       <c r="F6" s="2">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>82.88</v>
       </c>
       <c r="G6" s="2">
@@ -1811,136 +1811,136 @@
         <v>86.88</v>
       </c>
       <c r="H6" s="1">
-        <f>(E6-F6)/E6</f>
+        <f t="shared" si="1"/>
         <v>0.17120000000000005</v>
       </c>
       <c r="I6" s="1">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.13120000000000004</v>
       </c>
       <c r="J6" s="1">
         <v>13</v>
       </c>
       <c r="K6" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>12.959999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>2048</v>
       </c>
       <c r="C7" s="1">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="D7" s="1">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="E7" s="1">
+        <f t="shared" si="5"/>
+        <v>214</v>
+      </c>
+      <c r="F7" s="2">
+        <f t="shared" si="2"/>
+        <v>182.4</v>
+      </c>
+      <c r="G7" s="2">
+        <f t="shared" si="0"/>
+        <v>206.4</v>
+      </c>
+      <c r="H7" s="1">
+        <f t="shared" si="1"/>
+        <v>0.14766355140186913</v>
+      </c>
+      <c r="I7" s="1">
         <f t="shared" si="3"/>
-        <v>231</v>
-      </c>
-      <c r="F7" s="2">
-        <f t="shared" si="0"/>
-        <v>182.4</v>
-      </c>
-      <c r="G7" s="2">
-        <f>(2*B7/$A$2)*(1.04*LOG(B7/2,2)+1.5+IF(MOD(ROUND(K7,0)-1,3)=0,0,1))</f>
-        <v>206.4</v>
-      </c>
-      <c r="H7" s="1">
-        <f>(E7-F7)/E7</f>
-        <v>0.21038961038961038</v>
-      </c>
-      <c r="I7" s="1">
-        <f t="shared" si="1"/>
-        <v>0.10649350649350647</v>
+        <v>3.551401869158876E-2</v>
       </c>
       <c r="J7" s="1">
         <v>15</v>
       </c>
       <c r="K7" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>14.399999999999999</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>4096</v>
       </c>
       <c r="C8" s="1">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D8" s="1">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="E8" s="1">
+        <f t="shared" si="5"/>
+        <v>444</v>
+      </c>
+      <c r="F8" s="2">
+        <f t="shared" si="2"/>
+        <v>398.08000000000004</v>
+      </c>
+      <c r="G8" s="2">
+        <f t="shared" si="0"/>
+        <v>414.08000000000004</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" si="1"/>
+        <v>0.10342342342342332</v>
+      </c>
+      <c r="I8" s="1">
         <f t="shared" si="3"/>
-        <v>446</v>
-      </c>
-      <c r="F8" s="2">
-        <f t="shared" si="0"/>
-        <v>398.08000000000004</v>
-      </c>
-      <c r="G8" s="2">
-        <f>(2*B8/$A$2)*(1.04*LOG(B8/2,2)+1.5+IF(MOD(ROUND(K8,0)-1,3)=0,0,1))</f>
-        <v>414.08000000000004</v>
-      </c>
-      <c r="H8" s="1">
-        <f>(E8-F8)/E8</f>
-        <v>0.10744394618834072</v>
-      </c>
-      <c r="I8" s="1">
-        <f t="shared" si="1"/>
-        <v>7.1569506726457302E-2</v>
+        <v>6.7387387387387296E-2</v>
       </c>
       <c r="J8" s="1">
         <v>16</v>
       </c>
       <c r="K8" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>15.84</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>8192</v>
       </c>
       <c r="C9" s="1">
-        <v>510</v>
+        <v>480</v>
       </c>
       <c r="D9" s="1">
-        <v>475</v>
+        <v>446</v>
       </c>
       <c r="E9" s="1">
+        <f t="shared" si="5"/>
+        <v>926</v>
+      </c>
+      <c r="F9" s="2">
+        <f t="shared" si="2"/>
+        <v>862.72</v>
+      </c>
+      <c r="G9" s="2">
+        <f t="shared" si="0"/>
+        <v>958.72</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" si="1"/>
+        <v>6.8336933045356346E-2</v>
+      </c>
+      <c r="I9" s="1">
         <f t="shared" si="3"/>
-        <v>985</v>
-      </c>
-      <c r="F9" s="2">
-        <f t="shared" si="0"/>
-        <v>862.72</v>
-      </c>
-      <c r="G9" s="2">
-        <f>(2*B9/$A$2)*(1.04*LOG(B9/2,2)+1.5+IF(MOD(ROUND(K9,0)-1,3)=0,0,1))</f>
-        <v>958.72</v>
-      </c>
-      <c r="H9" s="1">
-        <f>(E9-F9)/E9</f>
-        <v>0.1241421319796954</v>
-      </c>
-      <c r="I9" s="1">
-        <f t="shared" si="1"/>
-        <v>2.668020304568525E-2</v>
+        <v>-3.533477321814258E-2</v>
       </c>
       <c r="J9" s="1">
         <v>17</v>
       </c>
       <c r="K9" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>17.28</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <f>8192*2</f>
         <v>16384</v>
@@ -1952,264 +1952,271 @@
         <v>974</v>
       </c>
       <c r="E10" s="1">
+        <f t="shared" si="5"/>
+        <v>2014</v>
+      </c>
+      <c r="F10" s="2">
+        <f t="shared" si="2"/>
+        <v>1858.56</v>
+      </c>
+      <c r="G10" s="2">
+        <f t="shared" si="0"/>
+        <v>1922.56</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="1"/>
+        <v>7.7179741807348587E-2</v>
+      </c>
+      <c r="I10" s="1">
         <f t="shared" si="3"/>
-        <v>2014</v>
-      </c>
-      <c r="F10" s="2">
-        <f t="shared" si="0"/>
-        <v>1858.56</v>
-      </c>
-      <c r="G10" s="2">
-        <f>(2*B10/$A$2)*(1.04*LOG(B10/2,2)+1.5+IF(MOD(ROUND(K10,0)-1,3)=0,0,1))</f>
-        <v>1922.56</v>
-      </c>
-      <c r="H10" s="1">
-        <f>(E10-F10)/E10</f>
-        <v>7.7179741807348587E-2</v>
-      </c>
-      <c r="I10" s="1">
-        <f t="shared" si="1"/>
         <v>4.5402184707050673E-2</v>
       </c>
       <c r="J10" s="1">
         <v>19</v>
       </c>
       <c r="K10" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>18.72</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <f>2*B10</f>
         <v>32768</v>
       </c>
       <c r="C11" s="1">
-        <v>2285</v>
+        <v>2158</v>
       </c>
       <c r="D11" s="1">
-        <v>2154</v>
+        <v>2028</v>
       </c>
       <c r="E11" s="1">
+        <f t="shared" si="5"/>
+        <v>4186</v>
+      </c>
+      <c r="F11" s="2">
+        <f t="shared" si="2"/>
+        <v>3983.36</v>
+      </c>
+      <c r="G11" s="2">
+        <f t="shared" si="0"/>
+        <v>4367.3600000000006</v>
+      </c>
+      <c r="H11" s="1">
+        <f t="shared" si="1"/>
+        <v>4.840898232202577E-2</v>
+      </c>
+      <c r="I11" s="1">
         <f t="shared" si="3"/>
-        <v>4439</v>
-      </c>
-      <c r="F11" s="2">
-        <f t="shared" si="0"/>
-        <v>3983.36</v>
-      </c>
-      <c r="G11" s="2">
-        <f>(2*B11/$A$2)*(1.04*LOG(B11/2,2)+1.5+IF(MOD(ROUND(K11,0)-1,3)=0,0,1))</f>
-        <v>4367.3600000000006</v>
-      </c>
-      <c r="H11" s="1">
-        <f>(E11-F11)/E11</f>
-        <v>0.10264473980626264</v>
-      </c>
-      <c r="I11" s="1">
-        <f t="shared" si="1"/>
-        <v>1.613876999324159E-2</v>
+        <v>-4.3325370281892157E-2</v>
       </c>
       <c r="J11" s="1">
         <v>20</v>
       </c>
       <c r="K11" s="1">
+        <f t="shared" si="4"/>
+        <v>20.16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B12" s="1">
+        <f t="shared" ref="B12:B16" si="6">2*B11</f>
+        <v>65536</v>
+      </c>
+      <c r="C12" s="1">
+        <v>4666</v>
+      </c>
+      <c r="D12" s="1">
+        <v>4408</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="5"/>
+        <v>9074</v>
+      </c>
+      <c r="F12" s="2">
         <f t="shared" si="2"/>
-        <v>20.16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="1">
-        <f t="shared" ref="B12:B16" si="4">2*B11</f>
-        <v>65536</v>
-      </c>
-      <c r="C12" s="1">
-        <v>4668</v>
-      </c>
-      <c r="D12" s="1">
-        <v>4410</v>
-      </c>
-      <c r="E12" s="1">
+        <v>8499.2000000000007</v>
+      </c>
+      <c r="G12" s="2">
+        <f t="shared" si="0"/>
+        <v>8755.2000000000007</v>
+      </c>
+      <c r="H12" s="1">
+        <f t="shared" si="1"/>
+        <v>6.3345823231209977E-2</v>
+      </c>
+      <c r="I12" s="1">
         <f t="shared" si="3"/>
-        <v>9078</v>
-      </c>
-      <c r="F12" s="2">
-        <f t="shared" si="0"/>
-        <v>8499.2000000000007</v>
-      </c>
-      <c r="G12" s="2">
-        <f>(2*B12/$A$2)*(1.04*LOG(B12/2,2)+1.5+IF(MOD(ROUND(K12,0)-1,3)=0,0,1))</f>
-        <v>8755.2000000000007</v>
-      </c>
-      <c r="H12" s="1">
-        <f>(E12-F12)/E12</f>
-        <v>6.3758537122714176E-2</v>
-      </c>
-      <c r="I12" s="1">
-        <f t="shared" si="1"/>
-        <v>3.555849306014533E-2</v>
+        <v>3.5133348027330757E-2</v>
       </c>
       <c r="J12" s="1">
         <v>22</v>
       </c>
       <c r="K12" s="1">
+        <f t="shared" si="4"/>
+        <v>21.599999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B13" s="1">
+        <f t="shared" si="6"/>
+        <v>131072</v>
+      </c>
+      <c r="C13" s="1">
+        <v>9714</v>
+      </c>
+      <c r="D13" s="1">
+        <v>9200</v>
+      </c>
+      <c r="E13" s="1">
+        <f t="shared" si="5"/>
+        <v>18914</v>
+      </c>
+      <c r="F13" s="2">
         <f t="shared" si="2"/>
-        <v>21.599999999999998</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B13" s="1">
-        <f t="shared" si="4"/>
-        <v>131072</v>
-      </c>
-      <c r="C13" s="1">
-        <v>10222</v>
-      </c>
-      <c r="D13" s="1">
-        <v>9707</v>
-      </c>
-      <c r="E13" s="1">
+        <v>18063.36</v>
+      </c>
+      <c r="G13" s="2">
+        <f t="shared" si="0"/>
+        <v>19599.36</v>
+      </c>
+      <c r="H13" s="1">
+        <f t="shared" si="1"/>
+        <v>4.4974093264248671E-2</v>
+      </c>
+      <c r="I13" s="1">
         <f t="shared" si="3"/>
-        <v>19929</v>
-      </c>
-      <c r="F13" s="2">
-        <f t="shared" si="0"/>
-        <v>18063.36</v>
-      </c>
-      <c r="G13" s="2">
-        <f>(2*B13/$A$2)*(1.04*LOG(B13/2,2)+1.5+IF(MOD(ROUND(K13,0)-1,3)=0,0,1))</f>
-        <v>19599.36</v>
-      </c>
-      <c r="H13" s="1">
-        <f>(E13-F13)/E13</f>
-        <v>9.3614330874604815E-2</v>
-      </c>
-      <c r="I13" s="1">
-        <f t="shared" si="1"/>
-        <v>1.6540719554418156E-2</v>
+        <v>-3.6235592682668953E-2</v>
       </c>
       <c r="J13" s="1">
         <v>23</v>
       </c>
       <c r="K13" s="1">
+        <f t="shared" si="4"/>
+        <v>23.04</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B14" s="1">
+        <f t="shared" si="6"/>
+        <v>262144</v>
+      </c>
+      <c r="C14" s="1">
+        <v>20830</v>
+      </c>
+      <c r="D14" s="1">
+        <v>19804</v>
+      </c>
+      <c r="E14" s="1">
+        <f>SUM(C14:D14)</f>
+        <v>40634</v>
+      </c>
+      <c r="F14" s="2">
         <f t="shared" si="2"/>
-        <v>23.04</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="1">
-        <f t="shared" si="4"/>
-        <v>262144</v>
-      </c>
-      <c r="C14" s="1">
-        <v>20828</v>
-      </c>
-      <c r="D14" s="1">
-        <v>19802</v>
-      </c>
-      <c r="E14" s="1">
+        <v>38256.639999999999</v>
+      </c>
+      <c r="G14" s="2">
+        <f t="shared" si="0"/>
+        <v>41328.639999999999</v>
+      </c>
+      <c r="H14" s="1">
+        <f t="shared" si="1"/>
+        <v>5.8506669291726154E-2</v>
+      </c>
+      <c r="I14" s="1">
         <f t="shared" si="3"/>
-        <v>40630</v>
-      </c>
-      <c r="F14" s="2">
-        <f t="shared" si="0"/>
-        <v>38256.639999999999</v>
-      </c>
-      <c r="G14" s="2">
-        <f>(2*B14/$A$2)*(1.04*LOG(B14/2,2)+1.5+IF(MOD(ROUND(K14,0)-1,3)=0,0,1))</f>
-        <v>41328.639999999999</v>
-      </c>
-      <c r="H14" s="1">
-        <f>(E14-F14)/E14</f>
-        <v>5.8413979817868583E-2</v>
-      </c>
-      <c r="I14" s="1">
-        <f t="shared" si="1"/>
-        <v>-1.7195175978341113E-2</v>
+        <v>-1.7095043559580633E-2</v>
       </c>
       <c r="J14" s="1">
         <v>25</v>
       </c>
       <c r="K14" s="1">
+        <f t="shared" si="4"/>
+        <v>24.48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B15" s="1">
+        <f t="shared" si="6"/>
+        <v>524288</v>
+      </c>
+      <c r="C15" s="1">
+        <v>43258</v>
+      </c>
+      <c r="D15" s="1">
+        <v>41208</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="5"/>
+        <v>84466</v>
+      </c>
+      <c r="F15" s="2">
         <f t="shared" si="2"/>
-        <v>24.48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B15" s="1">
-        <f t="shared" si="4"/>
-        <v>524288</v>
-      </c>
-      <c r="C15" s="1">
-        <v>45308</v>
-      </c>
-      <c r="D15" s="1">
-        <v>43257</v>
-      </c>
-      <c r="E15" s="1">
+        <v>80773.119999999995</v>
+      </c>
+      <c r="G15" s="2">
+        <f t="shared" si="0"/>
+        <v>86917.119999999995</v>
+      </c>
+      <c r="H15" s="1">
+        <f t="shared" si="1"/>
+        <v>4.3720313498922699E-2</v>
+      </c>
+      <c r="I15" s="1">
         <f t="shared" si="3"/>
-        <v>88565</v>
-      </c>
-      <c r="F15" s="2">
-        <f t="shared" si="0"/>
-        <v>80773.119999999995</v>
-      </c>
-      <c r="G15" s="2">
-        <f>(2*B15/$A$2)*(1.04*LOG(B15/2,2)+1.5+IF(MOD(ROUND(K15,0)-1,3)=0,0,1))</f>
-        <v>86917.119999999995</v>
-      </c>
-      <c r="H15" s="1">
-        <f>(E15-F15)/E15</f>
-        <v>8.7979224298537856E-2</v>
-      </c>
-      <c r="I15" s="1">
-        <f t="shared" si="1"/>
-        <v>1.8606447242138596E-2</v>
+        <v>-2.901901356758927E-2</v>
       </c>
       <c r="J15" s="1">
         <v>26</v>
       </c>
       <c r="K15" s="1">
+        <f t="shared" si="4"/>
+        <v>25.919999999999998</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B16" s="1">
+        <f t="shared" si="6"/>
+        <v>1048576</v>
+      </c>
+      <c r="C16" s="1">
+        <v>91833</v>
+      </c>
+      <c r="D16" s="1">
+        <v>87785</v>
+      </c>
+      <c r="E16" s="1">
+        <f t="shared" si="5"/>
+        <v>179618</v>
+      </c>
+      <c r="F16" s="2">
         <f t="shared" si="2"/>
-        <v>25.919999999999998</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B16" s="1">
-        <f t="shared" si="4"/>
-        <v>1048576</v>
-      </c>
-      <c r="E16" s="1">
+        <v>170065.92000000001</v>
+      </c>
+      <c r="G16" s="2">
+        <f t="shared" si="0"/>
+        <v>182353.92000000001</v>
+      </c>
+      <c r="H16" s="1">
+        <f t="shared" si="1"/>
+        <v>5.3179970826977181E-2</v>
+      </c>
+      <c r="I16" s="1">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="F16" s="2">
-        <f t="shared" si="0"/>
-        <v>170065.92000000001</v>
-      </c>
-      <c r="G16" s="2">
-        <f>(2*B16/$A$2)*(1.04*LOG(B16/2,2)+1.5+IF(MOD(ROUND(K16,0)-1,3)=0,0,1))</f>
-        <v>182353.92000000001</v>
-      </c>
-      <c r="H16" s="1" t="e">
-        <f>(E16-F16)/E16</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I16" s="1" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>-1.5231880991882845E-2</v>
       </c>
       <c r="J16" s="1"/>
       <c r="K16" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>27.36</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="E2:E9" formulaRange="1"/>
   </ignoredErrors>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>